<commit_message>
fix(admin): remove template guidance banner
</commit_message>
<xml_diff>
--- a/ui_kits/student/public/templates/job-import-template.xlsx
+++ b/ui_kits/student/public/templates/job-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="岗位数据" sheetId="1" r:id="R43d5be3abfa24d31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="R104bd9fac7844bd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="岗位数据" sheetId="1" r:id="Rcc5c1376aa12475b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="Ra8eaff238982450e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -242,7 +242,7 @@
         <x:color rgb="FFA61F34"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCECEF"/>
         </x:patternFill>
       </x:fill>
@@ -7439,16 +7439,15 @@
       <x:c r="E2" s="16"/>
       <x:c r="F2" s="16"/>
     </x:row>
-    <x:row r="3" ht="52" customHeight="1">
-      <x:c r="A3" s="25" t="str">
-        <x:v>请在“岗位数据”工作表中填写：第1行为固定表头，每行填写一个岗位；不要修改表头或合并单元格。导入成功后岗位会先进入草稿箱，请核对后再发布。大实习、小实习等类型仅作为参考，请按实际岗位选择。“薪资是否公开”选择“是”时，填写的薪资才会在岗位详情中展示。</x:v>
-      </x:c>
-      <x:c r="B3" s="26"/>
-      <x:c r="C3" s="26"/>
-      <x:c r="D3" s="26"/>
-      <x:c r="E3" s="26"/>
-      <x:c r="F3" s="27"/>
-    </x:row>
+    <x:row r="3" ht="8" customHeight="1">
+      <x:c r="A3"/>
+      <x:c r="B3"/>
+      <x:c r="C3"/>
+      <x:c r="D3"/>
+      <x:c r="E3"/>
+      <x:c r="F3"/>
+    </x:row>
+    <x:row r="4" ht="8" customHeight="1"/>
     <x:row r="5" ht="28" customHeight="1">
       <x:c r="A5" s="32" t="str">
         <x:v>列名</x:v>
@@ -8112,7 +8111,6 @@
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:F2"/>
-    <x:mergeCell ref="A3:F3"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="B6:B37">
     <x:cfRule type="expression" dxfId="0" priority="1">

</xml_diff>

<commit_message>
fix: refine required import fields
</commit_message>
<xml_diff>
--- a/ui_kits/student/public/templates/job-import-template.xlsx
+++ b/ui_kits/student/public/templates/job-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="岗位数据" sheetId="1" r:id="R566c464ac02f4432"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="Ra7cd2e6ba9904e8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="岗位数据" sheetId="1" r:id="R1257fafd135748b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="Rb84c6283b9cd40aa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -42,7 +42,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -62,6 +62,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFCFA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF332F2C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFA61F34"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -99,7 +109,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="21">
+  <x:cellXfs count="23">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -157,6 +167,12 @@
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -168,7 +184,7 @@
         <x:color rgb="FFA61F34"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFBEAEC"/>
         </x:patternFill>
       </x:fill>
@@ -406,88 +422,88 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="9" t="str">
+      <x:c r="A1" s="22" t="str">
         <x:v>单位名称</x:v>
       </x:c>
-      <x:c r="B1" s="8" t="str">
+      <x:c r="B1" s="21" t="str">
         <x:v>所属部门/业务线</x:v>
       </x:c>
-      <x:c r="C1" s="9" t="str">
+      <x:c r="C1" s="22" t="str">
         <x:v>岗位名称</x:v>
       </x:c>
-      <x:c r="D1" s="8" t="str">
+      <x:c r="D1" s="21" t="str">
         <x:v>招聘人数</x:v>
       </x:c>
-      <x:c r="E1" s="8" t="str">
+      <x:c r="E1" s="22" t="str">
         <x:v>岗位职责</x:v>
       </x:c>
-      <x:c r="F1" s="8" t="str">
+      <x:c r="F1" s="22" t="str">
         <x:v>招聘类型</x:v>
       </x:c>
-      <x:c r="G1" s="8" t="str">
+      <x:c r="G1" s="21" t="str">
         <x:v>工作形式</x:v>
       </x:c>
-      <x:c r="H1" s="8" t="str">
+      <x:c r="H1" s="21" t="str">
         <x:v>详细工作地点</x:v>
       </x:c>
-      <x:c r="I1" s="8" t="str">
+      <x:c r="I1" s="21" t="str">
         <x:v>投递截止日期</x:v>
       </x:c>
-      <x:c r="J1" s="9" t="str">
+      <x:c r="J1" s="22" t="str">
         <x:v>岗位大类</x:v>
       </x:c>
-      <x:c r="K1" s="8" t="str">
+      <x:c r="K1" s="21" t="str">
         <x:v>岗位小类</x:v>
       </x:c>
-      <x:c r="L1" s="8" t="str">
+      <x:c r="L1" s="21" t="str">
         <x:v>学历要求</x:v>
       </x:c>
-      <x:c r="M1" s="8" t="str">
+      <x:c r="M1" s="21" t="str">
         <x:v>工作开始日期</x:v>
       </x:c>
-      <x:c r="N1" s="8" t="str">
+      <x:c r="N1" s="21" t="str">
         <x:v>工作结束日期</x:v>
       </x:c>
-      <x:c r="O1" s="8" t="str">
+      <x:c r="O1" s="21" t="str">
         <x:v>工作省份</x:v>
       </x:c>
-      <x:c r="P1" s="8" t="str">
+      <x:c r="P1" s="21" t="str">
         <x:v>工作城市</x:v>
       </x:c>
-      <x:c r="Q1" s="8" t="str">
+      <x:c r="Q1" s="21" t="str">
         <x:v>每周天数（区间）</x:v>
       </x:c>
-      <x:c r="R1" s="8" t="str">
+      <x:c r="R1" s="21" t="str">
         <x:v>每周具体天数</x:v>
       </x:c>
-      <x:c r="S1" s="8" t="str">
+      <x:c r="S1" s="21" t="str">
         <x:v>实习时长</x:v>
       </x:c>
-      <x:c r="T1" s="8" t="str">
+      <x:c r="T1" s="22" t="str">
         <x:v>薪资是否公开</x:v>
       </x:c>
-      <x:c r="U1" s="8" t="str">
+      <x:c r="U1" s="21" t="str">
         <x:v>薪资下限（元/天）</x:v>
       </x:c>
-      <x:c r="V1" s="8" t="str">
+      <x:c r="V1" s="21" t="str">
         <x:v>薪资上限（元/天）</x:v>
       </x:c>
-      <x:c r="W1" s="8" t="str">
+      <x:c r="W1" s="21" t="str">
         <x:v>薪资展示文字</x:v>
       </x:c>
-      <x:c r="X1" s="8" t="str">
+      <x:c r="X1" s="21" t="str">
         <x:v>专业要求</x:v>
       </x:c>
-      <x:c r="Y1" s="8" t="str">
+      <x:c r="Y1" s="21" t="str">
         <x:v>毕业年份要求</x:v>
       </x:c>
-      <x:c r="Z1" s="8" t="str">
+      <x:c r="Z1" s="21" t="str">
         <x:v>技能要求</x:v>
       </x:c>
-      <x:c r="AA1" s="8" t="str">
+      <x:c r="AA1" s="21" t="str">
         <x:v>其他要求</x:v>
       </x:c>
-      <x:c r="AB1" s="8" t="str">
+      <x:c r="AB1" s="21" t="str">
         <x:v>官网投递链接</x:v>
       </x:c>
     </x:row>
@@ -6663,7 +6679,7 @@
         <x:v>岗位职责</x:v>
       </x:c>
       <x:c r="B10" s="20" t="str">
-        <x:v>选填</x:v>
+        <x:v>必填</x:v>
       </x:c>
       <x:c r="C10" s="16" t="str">
         <x:v>长文本</x:v>
@@ -6683,7 +6699,7 @@
         <x:v>招聘类型</x:v>
       </x:c>
       <x:c r="B11" s="20" t="str">
-        <x:v>选填</x:v>
+        <x:v>必填</x:v>
       </x:c>
       <x:c r="C11" s="16" t="str">
         <x:v>下拉选项</x:v>
@@ -6963,7 +6979,7 @@
         <x:v>薪资是否公开</x:v>
       </x:c>
       <x:c r="B25" s="20" t="str">
-        <x:v>选填</x:v>
+        <x:v>必填</x:v>
       </x:c>
       <x:c r="C25" s="16" t="str">
         <x:v>下拉选项</x:v>

</xml_diff>